<commit_message>
Fix maintenance schedule signature placeholders
</commit_message>
<xml_diff>
--- a/resources/templates/maintenance-annual-template.xlsx
+++ b/resources/templates/maintenance-annual-template.xlsx
@@ -43,7 +43,7 @@
     <t>_________________________</t>
   </si>
   <si>
-    <t>А.А.Королев</t>
+    <t/>
   </si>
   <si>
     <t>ГОДОВОЙ ГРАФИК</t>
@@ -216,7 +216,7 @@
     <t>Начальник КЦ</t>
   </si>
   <si>
-    <t>М.И.Малашкеевич</t>
+    <t/>
   </si>
   <si>
     <t>СОГЛАСОВАНО</t>

</xml_diff>